<commit_message>
refactor(structure): Align project with submission file structure
- Refactored core logic into the required directory structure.
- Moved EventRegistry and upcasters to src/upcasting/.
- Moved audit chain logic to src/integrity/.
- Moved MCP server to src/mcp/server.py and created tools.py and resources.py.
- Created formal command models and handlers in src/commands/.
- Renamed projection files to match specification.
</commit_message>
<xml_diff>
--- a/documents/COMP-001/financial_statements.xlsx
+++ b/documents/COMP-001/financial_statements.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Income Statement" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Key Ratios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Ratios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>